<commit_message>
Emergency Due Settlement Page
</commit_message>
<xml_diff>
--- a/InputData/DataProvider_FrontOffice.xlsx
+++ b/InputData/DataProvider_FrontOffice.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D7C8F4C-FC34-408A-A54B-331799C6C444}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E6DC503-D929-4993-97E2-6B4476A3E150}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="84" activeTab="86" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="92" activeTab="93" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FO_Registration_Page" sheetId="15" r:id="rId1"/>
@@ -67,34 +67,41 @@
     <sheet name="IP_Billing_Audit_Clearance" sheetId="74" r:id="rId57"/>
     <sheet name="Acknowledge_Discharge_Page" sheetId="75" r:id="rId58"/>
     <sheet name="MiscellaneousCharges_Page" sheetId="76" r:id="rId59"/>
-    <sheet name="Ip_Ambulance_MrdCharges" sheetId="77" r:id="rId60"/>
-    <sheet name="IP_Pending_Investigation" sheetId="78" r:id="rId61"/>
-    <sheet name="IP_Credit_Limit" sheetId="79" r:id="rId62"/>
-    <sheet name="IP_General_OrderEntry" sheetId="80" r:id="rId63"/>
-    <sheet name="Ip_Doctor_Vist_Page" sheetId="86" r:id="rId64"/>
-    <sheet name="Ip_Billing_Page" sheetId="87" r:id="rId65"/>
-    <sheet name="Ip_Bill_Add_on_Bill" sheetId="89" r:id="rId66"/>
-    <sheet name="Due_Settlement_Page" sheetId="90" r:id="rId67"/>
-    <sheet name="Ip_DepositRefund_Page" sheetId="91" r:id="rId68"/>
-    <sheet name="Ip_Refund_Page" sheetId="92" r:id="rId69"/>
-    <sheet name="Ip_ReceiptUtility_Page" sheetId="93" r:id="rId70"/>
-    <sheet name="OP_Deposit_Transfer_Ip" sheetId="94" r:id="rId71"/>
-    <sheet name="IP_Cheque_In_HandDetails" sheetId="95" r:id="rId72"/>
-    <sheet name="IP_Cheque_In_Hand" sheetId="96" r:id="rId73"/>
-    <sheet name="Package_Modifiction_Patient_Pag" sheetId="98" r:id="rId74"/>
-    <sheet name="ADT_Package_Multiple" sheetId="99" r:id="rId75"/>
-    <sheet name="Package_Duration_Modifiction" sheetId="97" r:id="rId76"/>
-    <sheet name="Nursing_Clearance_Page" sheetId="81" r:id="rId77"/>
-    <sheet name="Nursing_Activity_Page" sheetId="85" r:id="rId78"/>
-    <sheet name="Pharmacy_Discharge_Notification" sheetId="83" r:id="rId79"/>
-    <sheet name="Lab_Clearance_Page" sheetId="84" r:id="rId80"/>
-    <sheet name="ER_Registration_Page" sheetId="100" r:id="rId81"/>
-    <sheet name="ER_To_Admit_Sheet" sheetId="101" r:id="rId82"/>
-    <sheet name="Er_Activity_Sheet" sheetId="102" r:id="rId83"/>
-    <sheet name="Er_Admission_Update_DateTime" sheetId="103" r:id="rId84"/>
-    <sheet name="Er_Admission_Surgery_Request" sheetId="104" r:id="rId85"/>
-    <sheet name="Er_CreditLimitPage" sheetId="105" r:id="rId86"/>
-    <sheet name="Er_Billing_Page" sheetId="106" r:id="rId87"/>
+    <sheet name="Sheet1" sheetId="107" r:id="rId60"/>
+    <sheet name="Ip_Ambulance_MrdCharges" sheetId="77" r:id="rId61"/>
+    <sheet name="IP_Pending_Investigation" sheetId="78" r:id="rId62"/>
+    <sheet name="IP_Credit_Limit" sheetId="79" r:id="rId63"/>
+    <sheet name="IP_General_OrderEntry" sheetId="80" r:id="rId64"/>
+    <sheet name="Ip_Doctor_Vist_Page" sheetId="86" r:id="rId65"/>
+    <sheet name="Ip_Billing_Page" sheetId="87" r:id="rId66"/>
+    <sheet name="Ip_Bill_Add_on_Bill" sheetId="89" r:id="rId67"/>
+    <sheet name="Due_Settlement_Page" sheetId="90" r:id="rId68"/>
+    <sheet name="Ip_DepositRefund_Page" sheetId="91" r:id="rId69"/>
+    <sheet name="Ip_Refund_Page" sheetId="92" r:id="rId70"/>
+    <sheet name="Ip_ReceiptUtility_Page" sheetId="93" r:id="rId71"/>
+    <sheet name="OP_Deposit_Transfer_Ip" sheetId="94" r:id="rId72"/>
+    <sheet name="IP_Cheque_In_HandDetails" sheetId="95" r:id="rId73"/>
+    <sheet name="IP_Cheque_In_Hand" sheetId="96" r:id="rId74"/>
+    <sheet name="Package_Modifiction_Patient_Pag" sheetId="98" r:id="rId75"/>
+    <sheet name="ADT_Package_Multiple" sheetId="99" r:id="rId76"/>
+    <sheet name="Package_Duration_Modifiction" sheetId="97" r:id="rId77"/>
+    <sheet name="Nursing_Clearance_Page" sheetId="81" r:id="rId78"/>
+    <sheet name="Nursing_Activity_Page" sheetId="85" r:id="rId79"/>
+    <sheet name="Pharmacy_Discharge_Notification" sheetId="83" r:id="rId80"/>
+    <sheet name="Lab_Clearance_Page" sheetId="84" r:id="rId81"/>
+    <sheet name="ER_Registration_Page" sheetId="100" r:id="rId82"/>
+    <sheet name="ER_To_Admit_Sheet" sheetId="101" r:id="rId83"/>
+    <sheet name="Er_Activity_Sheet" sheetId="102" r:id="rId84"/>
+    <sheet name="Er_Admission_Update_DateTime" sheetId="103" r:id="rId85"/>
+    <sheet name="Er_Admission_Surgery_Request" sheetId="104" r:id="rId86"/>
+    <sheet name="Er_CreditLimitPage" sheetId="105" r:id="rId87"/>
+    <sheet name="Er_Billing_Page" sheetId="106" r:id="rId88"/>
+    <sheet name="Er_MiscellaneousCharges_Page" sheetId="108" r:id="rId89"/>
+    <sheet name="Er_AmbulanceCharges_Page" sheetId="109" r:id="rId90"/>
+    <sheet name="Er_TOC_Approval_Page" sheetId="110" r:id="rId91"/>
+    <sheet name="Er_Discharge_Notification_Page" sheetId="111" r:id="rId92"/>
+    <sheet name="Er_DueSettlement_Page" sheetId="113" r:id="rId93"/>
+    <sheet name="Er_DepositRefund_Page" sheetId="114" r:id="rId94"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -106,7 +113,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2409" uniqueCount="1352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2507" uniqueCount="1380">
   <si>
     <t>SANITY HOSPITAL</t>
   </si>
@@ -4162,6 +4169,90 @@
   </si>
   <si>
     <t xml:space="preserve">Anup </t>
+  </si>
+  <si>
+    <t>Amount_enter</t>
+  </si>
+  <si>
+    <t>Dr.Employee102</t>
+  </si>
+  <si>
+    <t>SPSL.886318</t>
+  </si>
+  <si>
+    <t>Name_Search_Medical_Record_Charges</t>
+  </si>
+  <si>
+    <t>Admission Fees</t>
+  </si>
+  <si>
+    <t>Remark</t>
+  </si>
+  <si>
+    <t>Search_TOC_Approved_From_Date</t>
+  </si>
+  <si>
+    <t>Search_TOC_Approved_To_Date</t>
+  </si>
+  <si>
+    <t>Cancel Remarks Bill</t>
+  </si>
+  <si>
+    <t>Cancel_Bill_Reamrks</t>
+  </si>
+  <si>
+    <t>Status_DropDwon</t>
+  </si>
+  <si>
+    <t>Patient_Type_Drp</t>
+  </si>
+  <si>
+    <t>Discharge</t>
+  </si>
+  <si>
+    <t>ER NO</t>
+  </si>
+  <si>
+    <t>Find_Patient_Frome_Date</t>
+  </si>
+  <si>
+    <t>Enter_Due_Amount_Er_Number</t>
+  </si>
+  <si>
+    <t>Enter_Rounding_Off_Settlement</t>
+  </si>
+  <si>
+    <t>Remarks_Due_Settlement</t>
+  </si>
+  <si>
+    <t>Anup Due Settlement</t>
+  </si>
+  <si>
+    <t>Enter_Cheque_Number</t>
+  </si>
+  <si>
+    <t>Less_Amount_Due_Amount</t>
+  </si>
+  <si>
+    <t>Serach_Company_Frome_Date</t>
+  </si>
+  <si>
+    <t>Serach_Company_To_Date</t>
+  </si>
+  <si>
+    <t>Deposit_Case_Amount</t>
+  </si>
+  <si>
+    <t>Deposit_Remarks</t>
+  </si>
+  <si>
+    <t>Relationship_Drp</t>
+  </si>
+  <si>
+    <t>Deposit_Cheque_Amount</t>
+  </si>
+  <si>
+    <t>Deposit_Er_Number</t>
   </si>
 </sst>
 </file>
@@ -4228,7 +4319,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -4242,6 +4333,7 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -11356,6 +11448,15 @@
 </file>
 
 <file path=xl/worksheets/sheet60.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C888D81-EFB3-4567-80FC-3EBB12959E54}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{524359A0-2104-4284-80DF-E4D467856F6E}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -11420,7 +11521,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{658E2525-34D4-493E-BC75-42FCB8785136}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -11493,7 +11594,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5D44066-CCF8-4E69-8974-47BB22EA7B20}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -11550,7 +11651,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D536C2E-2049-4378-975D-D0690C151CB0}">
   <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -11671,7 +11772,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{869035F4-0440-4683-84DA-B1D3A25F3843}">
   <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -11785,7 +11886,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8FB2B9F-5C63-4573-B0FF-F4AA329DC337}">
   <dimension ref="A1:BC2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -12185,7 +12286,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D418190-A307-409C-9B13-520CE3406CF2}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -12208,7 +12309,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EB81613-B25D-46A1-9C96-7C4B253B73B9}">
   <dimension ref="A1:AO2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -12508,7 +12609,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3883C6CD-3A6E-4057-B81E-312B0FC40198}">
   <dimension ref="A1:AI2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -12769,7 +12870,72 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4E25BFB-5A64-45CB-AFD0-C13AA2181D17}">
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="34.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" t="s">
+        <v>718</v>
+      </c>
+      <c r="D1" t="s">
+        <v>719</v>
+      </c>
+      <c r="E1" t="s">
+        <v>720</v>
+      </c>
+      <c r="F1" t="s">
+        <v>721</v>
+      </c>
+      <c r="G1" t="s">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C2" t="s">
+        <v>726</v>
+      </c>
+      <c r="D2" t="s">
+        <v>723</v>
+      </c>
+      <c r="E2" t="s">
+        <v>724</v>
+      </c>
+      <c r="F2" s="1">
+        <v>46043</v>
+      </c>
+      <c r="G2" t="s">
+        <v>725</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet70.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E1F95AA-9032-47A7-9B12-71766439ACDD}">
   <dimension ref="A1:AH2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -13019,72 +13185,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4E25BFB-5A64-45CB-AFD0-C13AA2181D17}">
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="34.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="31.28515625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1" t="s">
-        <v>718</v>
-      </c>
-      <c r="D1" t="s">
-        <v>719</v>
-      </c>
-      <c r="E1" t="s">
-        <v>720</v>
-      </c>
-      <c r="F1" t="s">
-        <v>721</v>
-      </c>
-      <c r="G1" t="s">
-        <v>722</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>106</v>
-      </c>
-      <c r="C2" t="s">
-        <v>726</v>
-      </c>
-      <c r="D2" t="s">
-        <v>723</v>
-      </c>
-      <c r="E2" t="s">
-        <v>724</v>
-      </c>
-      <c r="F2" s="1">
-        <v>46043</v>
-      </c>
-      <c r="G2" t="s">
-        <v>725</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet70.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD618DE6-3AFD-4017-B22F-08C9D50DAA49}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -13142,7 +13243,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E58E864-6E8A-4FF7-945A-7E806EFB2D6C}">
   <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -13222,7 +13323,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4077AA7E-88E2-4256-86EA-52919803DDCC}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -13267,7 +13368,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet74.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A1A5E74-AAFE-4352-879F-C9ADB66D4324}">
   <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -13367,7 +13468,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet74.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet75.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54354EAF-1340-4149-90BD-A72ECC03E494}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -13424,7 +13525,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet75.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet76.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4ECF30F3-2043-4C80-AFAE-88161DDB3A16}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -13482,7 +13583,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet76.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet77.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A989A04-A33E-4EEF-912B-E0583A70A2FD}">
   <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -13561,7 +13662,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet77.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet78.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12F09270-1FEE-4D7E-A2B1-067B6E58EC0B}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -13633,7 +13734,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet78.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet79.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1B73523-0C7D-4155-AC44-E87812CD37B8}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -13677,85 +13778,6 @@
       </c>
       <c r="E2" t="s">
         <v>996</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet79.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48C6946A-E358-4DE2-B43D-AD5F7808634C}">
-  <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="30.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="28.7109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>900</v>
-      </c>
-      <c r="B1" t="s">
-        <v>979</v>
-      </c>
-      <c r="C1" t="s">
-        <v>919</v>
-      </c>
-      <c r="D1" t="s">
-        <v>981</v>
-      </c>
-      <c r="E1" t="s">
-        <v>975</v>
-      </c>
-      <c r="F1" t="s">
-        <v>976</v>
-      </c>
-      <c r="G1" t="s">
-        <v>951</v>
-      </c>
-      <c r="H1" t="s">
-        <v>977</v>
-      </c>
-      <c r="I1" t="s">
-        <v>978</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>980</v>
-      </c>
-      <c r="C2" t="s">
-        <v>523</v>
-      </c>
-      <c r="D2" t="s">
-        <v>523</v>
-      </c>
-      <c r="E2" s="1">
-        <v>46054</v>
-      </c>
-      <c r="F2" t="s">
-        <v>848</v>
-      </c>
-      <c r="G2">
-        <v>29344</v>
-      </c>
-      <c r="H2" t="s">
-        <v>910</v>
-      </c>
-      <c r="I2" s="1">
-        <v>46057</v>
       </c>
     </row>
   </sheetData>
@@ -13836,6 +13858,85 @@
 </file>
 
 <file path=xl/worksheets/sheet80.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48C6946A-E358-4DE2-B43D-AD5F7808634C}">
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="28.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>900</v>
+      </c>
+      <c r="B1" t="s">
+        <v>979</v>
+      </c>
+      <c r="C1" t="s">
+        <v>919</v>
+      </c>
+      <c r="D1" t="s">
+        <v>981</v>
+      </c>
+      <c r="E1" t="s">
+        <v>975</v>
+      </c>
+      <c r="F1" t="s">
+        <v>976</v>
+      </c>
+      <c r="G1" t="s">
+        <v>951</v>
+      </c>
+      <c r="H1" t="s">
+        <v>977</v>
+      </c>
+      <c r="I1" t="s">
+        <v>978</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>980</v>
+      </c>
+      <c r="C2" t="s">
+        <v>523</v>
+      </c>
+      <c r="D2" t="s">
+        <v>523</v>
+      </c>
+      <c r="E2" s="1">
+        <v>46054</v>
+      </c>
+      <c r="F2" t="s">
+        <v>848</v>
+      </c>
+      <c r="G2">
+        <v>29344</v>
+      </c>
+      <c r="H2" t="s">
+        <v>910</v>
+      </c>
+      <c r="I2" s="1">
+        <v>46057</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet81.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2753D503-B7CA-43F7-BD19-60134A1E726F}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -13907,7 +14008,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet81.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet82.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9984DF16-1A75-4635-9101-206351EE1444}">
   <dimension ref="A1:CP2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -14561,7 +14662,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet82.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet83.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A30D36C-D939-4BE3-85F0-D947812190E5}">
   <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -14682,7 +14783,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet83.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet84.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6369E9D3-38E6-4C79-8ECA-0C7BD071C1A0}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -14745,7 +14846,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet84.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet85.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2297FC27-8B95-4994-AC55-7579464FE13D}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -14774,7 +14875,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet85.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet86.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F8BE78D-628E-45AA-BF42-043C9973B432}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -14839,7 +14940,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet86.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet87.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D228C6F9-C725-4AFE-A2CE-EEC08172626E}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -14889,7 +14990,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet87.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet88.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{617F797D-41D1-4D94-B217-DDA96A6A7FB3}">
   <dimension ref="A1:AF2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -15037,7 +15138,7 @@
         <v>46104</v>
       </c>
       <c r="E2">
-        <v>1508826</v>
+        <v>1508833</v>
       </c>
       <c r="F2" t="s">
         <v>214</v>
@@ -15124,6 +15225,99 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet89.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31373D41-CE00-4FCF-80C5-C80B936CA804}">
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="32.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="24.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>900</v>
+      </c>
+      <c r="B1" t="s">
+        <v>901</v>
+      </c>
+      <c r="C1" t="s">
+        <v>948</v>
+      </c>
+      <c r="D1" t="s">
+        <v>450</v>
+      </c>
+      <c r="E1" t="s">
+        <v>422</v>
+      </c>
+      <c r="F1" t="s">
+        <v>423</v>
+      </c>
+      <c r="G1" t="s">
+        <v>935</v>
+      </c>
+      <c r="H1" t="s">
+        <v>936</v>
+      </c>
+      <c r="I1" t="s">
+        <v>1352</v>
+      </c>
+      <c r="J1" t="s">
+        <v>940</v>
+      </c>
+      <c r="K1" t="s">
+        <v>934</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1219</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1354</v>
+      </c>
+      <c r="D2">
+        <v>1508832</v>
+      </c>
+      <c r="E2" s="1">
+        <v>46003</v>
+      </c>
+      <c r="F2" s="1">
+        <v>46108</v>
+      </c>
+      <c r="G2" t="s">
+        <v>945</v>
+      </c>
+      <c r="H2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2">
+        <v>400</v>
+      </c>
+      <c r="J2">
+        <v>2</v>
+      </c>
+      <c r="K2" t="s">
+        <v>1353</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -15155,4 +15349,470 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet90.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E91BB5C-5E49-4DB9-9FB9-44F7CC387A01}">
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="21" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="37.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>900</v>
+      </c>
+      <c r="B1" t="s">
+        <v>901</v>
+      </c>
+      <c r="C1" t="s">
+        <v>422</v>
+      </c>
+      <c r="D1" t="s">
+        <v>423</v>
+      </c>
+      <c r="E1" t="s">
+        <v>948</v>
+      </c>
+      <c r="F1" t="s">
+        <v>450</v>
+      </c>
+      <c r="G1" t="s">
+        <v>1355</v>
+      </c>
+      <c r="H1" t="s">
+        <v>956</v>
+      </c>
+      <c r="I1" t="s">
+        <v>1357</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1219</v>
+      </c>
+      <c r="C2" s="1">
+        <v>46101</v>
+      </c>
+      <c r="D2" s="1">
+        <v>46111</v>
+      </c>
+      <c r="E2" t="s">
+        <v>1354</v>
+      </c>
+      <c r="F2">
+        <v>1508832</v>
+      </c>
+      <c r="G2" t="s">
+        <v>1356</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+      <c r="I2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet91.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E09F33E-BC12-4F39-AE5B-A7CC7E51637E}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="32.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="30.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>900</v>
+      </c>
+      <c r="B1" t="s">
+        <v>901</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1336</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1358</v>
+      </c>
+      <c r="E1" t="s">
+        <v>1359</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1219</v>
+      </c>
+      <c r="C2">
+        <v>1508837</v>
+      </c>
+      <c r="D2" s="1">
+        <v>46111</v>
+      </c>
+      <c r="E2" s="1">
+        <v>46112</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet92.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA2505F4-A146-4541-AE1A-D1742769B6EE}">
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="32.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>900</v>
+      </c>
+      <c r="B1" t="s">
+        <v>901</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1361</v>
+      </c>
+      <c r="D1" t="s">
+        <v>919</v>
+      </c>
+      <c r="E1" t="s">
+        <v>1362</v>
+      </c>
+      <c r="F1" t="s">
+        <v>433</v>
+      </c>
+      <c r="G1" t="s">
+        <v>423</v>
+      </c>
+      <c r="H1" t="s">
+        <v>1363</v>
+      </c>
+      <c r="I1" t="s">
+        <v>1345</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1219</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1360</v>
+      </c>
+      <c r="D2" t="s">
+        <v>1258</v>
+      </c>
+      <c r="E2" t="s">
+        <v>1364</v>
+      </c>
+      <c r="F2" s="1">
+        <v>46109</v>
+      </c>
+      <c r="G2" s="1">
+        <v>46112</v>
+      </c>
+      <c r="H2" t="s">
+        <v>1365</v>
+      </c>
+      <c r="I2">
+        <v>1508804</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet93.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11B928DB-F65E-4332-B1DF-634D0E704CBC}">
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="28.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="30.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="24" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="30.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>900</v>
+      </c>
+      <c r="B1" t="s">
+        <v>901</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1366</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1163</v>
+      </c>
+      <c r="E1" t="s">
+        <v>424</v>
+      </c>
+      <c r="F1" t="s">
+        <v>1373</v>
+      </c>
+      <c r="G1" t="s">
+        <v>1374</v>
+      </c>
+      <c r="H1" t="s">
+        <v>1367</v>
+      </c>
+      <c r="I1" t="s">
+        <v>1371</v>
+      </c>
+      <c r="J1" t="s">
+        <v>497</v>
+      </c>
+      <c r="K1" t="s">
+        <v>242</v>
+      </c>
+      <c r="L1" t="s">
+        <v>499</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>1372</v>
+      </c>
+      <c r="N1" t="s">
+        <v>1368</v>
+      </c>
+      <c r="O1" t="s">
+        <v>1369</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1219</v>
+      </c>
+      <c r="C2" s="1">
+        <v>46112</v>
+      </c>
+      <c r="D2" s="1">
+        <v>46114</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="F2" s="1">
+        <v>46101</v>
+      </c>
+      <c r="G2" s="1">
+        <v>46114</v>
+      </c>
+      <c r="H2" s="13">
+        <v>1508851</v>
+      </c>
+      <c r="I2">
+        <v>123456</v>
+      </c>
+      <c r="J2" s="1">
+        <v>46114</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="M2" s="13">
+        <v>10</v>
+      </c>
+      <c r="N2">
+        <v>1</v>
+      </c>
+      <c r="O2" t="s">
+        <v>1370</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet94.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0C0EE80-01C8-4453-A92B-89D25A36D783}">
+  <dimension ref="A1:Q2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="32.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="24" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>900</v>
+      </c>
+      <c r="B1" t="s">
+        <v>901</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1366</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1163</v>
+      </c>
+      <c r="E1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" t="s">
+        <v>1336</v>
+      </c>
+      <c r="G1" t="s">
+        <v>1375</v>
+      </c>
+      <c r="H1" t="s">
+        <v>1376</v>
+      </c>
+      <c r="I1" t="s">
+        <v>1377</v>
+      </c>
+      <c r="J1" t="s">
+        <v>1378</v>
+      </c>
+      <c r="K1" t="s">
+        <v>537</v>
+      </c>
+      <c r="L1" t="s">
+        <v>497</v>
+      </c>
+      <c r="M1" t="s">
+        <v>242</v>
+      </c>
+      <c r="N1" t="s">
+        <v>499</v>
+      </c>
+      <c r="O1" t="s">
+        <v>1379</v>
+      </c>
+      <c r="P1" t="s">
+        <v>1167</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1219</v>
+      </c>
+      <c r="C2" s="1">
+        <v>46111</v>
+      </c>
+      <c r="D2" s="1">
+        <v>46114</v>
+      </c>
+      <c r="E2" t="s">
+        <v>1354</v>
+      </c>
+      <c r="F2">
+        <v>1508844</v>
+      </c>
+      <c r="G2">
+        <v>700</v>
+      </c>
+      <c r="H2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" t="s">
+        <v>16</v>
+      </c>
+      <c r="J2">
+        <v>800</v>
+      </c>
+      <c r="K2">
+        <v>123456</v>
+      </c>
+      <c r="L2" s="1">
+        <v>46114</v>
+      </c>
+      <c r="M2" t="s">
+        <v>1072</v>
+      </c>
+      <c r="N2" t="s">
+        <v>8</v>
+      </c>
+      <c r="O2">
+        <v>1508832</v>
+      </c>
+      <c r="P2" s="1">
+        <v>46114</v>
+      </c>
+      <c r="Q2" s="1">
+        <v>46115</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>